<commit_message>
Add PiN step 1 hybrid for Central_African_Republic___CAR
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Central_African_Republic___CAR/PiN_step1_Central_African_Republic___CAR_1008_03PM.xlsx
+++ b/platform_PiN_output/Central_African_Republic___CAR/PiN_step1_Central_African_Republic___CAR_1008_03PM.xlsx
@@ -1267,34 +1267,34 @@
         <v>1706</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>32.5</v>
+        <v>32.1</v>
       </c>
       <c r="E4" s="30" t="n">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="F4" s="30" t="n">
-        <v>53.7</v>
+        <v>49.3</v>
       </c>
       <c r="G4" s="30" t="n">
-        <v>916</v>
+        <v>841</v>
       </c>
       <c r="H4" s="30" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I4" s="30" t="n">
+        <v>98</v>
+      </c>
+      <c r="J4" s="30" t="n">
         <v>12.9</v>
       </c>
-      <c r="I4" s="30" t="n">
+      <c r="K4" s="30" t="n">
         <v>220</v>
       </c>
-      <c r="J4" s="30" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="K4" s="30" t="n">
-        <v>15</v>
-      </c>
       <c r="L4" s="30" t="n">
-        <v>67.5</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="M4" s="30" t="n">
-        <v>1151</v>
+        <v>1159</v>
       </c>
       <c r="N4" s="31" t="inlineStr">
         <is>
@@ -1435,34 +1435,34 @@
         <v>2134</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>61.3</v>
+        <v>60.9</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>1309</v>
+        <v>1300</v>
       </c>
       <c r="F5" s="30" t="n">
-        <v>28.9</v>
+        <v>29.3</v>
       </c>
       <c r="G5" s="30" t="n">
-        <v>617</v>
+        <v>626</v>
       </c>
       <c r="H5" s="30" t="n">
-        <v>8.4</v>
+        <v>4</v>
       </c>
       <c r="I5" s="30" t="n">
-        <v>180</v>
+        <v>85</v>
       </c>
       <c r="J5" s="30" t="n">
-        <v>1.3</v>
+        <v>5.8</v>
       </c>
       <c r="K5" s="30" t="n">
-        <v>28</v>
+        <v>123</v>
       </c>
       <c r="L5" s="30" t="n">
-        <v>38.7</v>
+        <v>39.1</v>
       </c>
       <c r="M5" s="30" t="n">
-        <v>825</v>
+        <v>835</v>
       </c>
       <c r="N5" s="31" t="inlineStr">
         <is>
@@ -1603,34 +1603,34 @@
         <v>5891</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>65.90000000000001</v>
+        <v>65</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>3882</v>
+        <v>3829</v>
       </c>
       <c r="F6" s="30" t="n">
-        <v>24.2</v>
+        <v>26.4</v>
       </c>
       <c r="G6" s="30" t="n">
-        <v>1424</v>
+        <v>1554</v>
       </c>
       <c r="H6" s="30" t="n">
-        <v>9.300000000000001</v>
+        <v>0</v>
       </c>
       <c r="I6" s="30" t="n">
-        <v>548</v>
+        <v>0</v>
       </c>
       <c r="J6" s="30" t="n">
-        <v>0.6</v>
+        <v>8.6</v>
       </c>
       <c r="K6" s="30" t="n">
-        <v>36</v>
+        <v>508</v>
       </c>
       <c r="L6" s="30" t="n">
-        <v>34.1</v>
+        <v>35</v>
       </c>
       <c r="M6" s="30" t="n">
-        <v>2008</v>
+        <v>2062</v>
       </c>
       <c r="N6" s="31" t="inlineStr">
         <is>
@@ -2329,22 +2329,22 @@
         <v>85</v>
       </c>
       <c r="F10" s="30" t="n">
-        <v>46</v>
+        <v>35.6</v>
       </c>
       <c r="G10" s="30" t="n">
-        <v>256</v>
+        <v>198</v>
       </c>
       <c r="H10" s="30" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="I10" s="30" t="n">
+        <v>61</v>
+      </c>
+      <c r="J10" s="30" t="n">
         <v>38</v>
       </c>
-      <c r="I10" s="30" t="n">
+      <c r="K10" s="30" t="n">
         <v>211</v>
-      </c>
-      <c r="J10" s="30" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="K10" s="30" t="n">
-        <v>4</v>
       </c>
       <c r="L10" s="30" t="n">
         <v>84.7</v>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="N10" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O10" s="32" t="n">
@@ -3035,38 +3035,38 @@
         <v>6561</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>55.4</v>
+        <v>53.2</v>
       </c>
       <c r="E14" s="30" t="n">
-        <v>3636</v>
+        <v>3491</v>
       </c>
       <c r="F14" s="30" t="n">
         <v>16.2</v>
       </c>
       <c r="G14" s="30" t="n">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="H14" s="30" t="n">
-        <v>28.3</v>
+        <v>9.9</v>
       </c>
       <c r="I14" s="30" t="n">
-        <v>1860</v>
+        <v>653</v>
       </c>
       <c r="J14" s="30" t="n">
-        <v>0</v>
+        <v>20.6</v>
       </c>
       <c r="K14" s="30" t="n">
-        <v>1</v>
+        <v>1353</v>
       </c>
       <c r="L14" s="30" t="n">
-        <v>44.6</v>
+        <v>46.8</v>
       </c>
       <c r="M14" s="30" t="n">
-        <v>2924</v>
+        <v>3069</v>
       </c>
       <c r="N14" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O14" s="32" t="n">
@@ -3213,34 +3213,34 @@
         <v>5670</v>
       </c>
       <c r="D15" s="30" t="n">
-        <v>60.3</v>
+        <v>59</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>3420</v>
+        <v>3348</v>
       </c>
       <c r="F15" s="30" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="G15" s="30" t="n">
-        <v>1027</v>
+        <v>1041</v>
       </c>
       <c r="H15" s="30" t="n">
-        <v>20.5</v>
+        <v>4.2</v>
       </c>
       <c r="I15" s="30" t="n">
-        <v>1164</v>
+        <v>235</v>
       </c>
       <c r="J15" s="30" t="n">
-        <v>1</v>
+        <v>18.4</v>
       </c>
       <c r="K15" s="30" t="n">
-        <v>59</v>
+        <v>1046</v>
       </c>
       <c r="L15" s="30" t="n">
-        <v>39.7</v>
+        <v>41</v>
       </c>
       <c r="M15" s="30" t="n">
-        <v>2251</v>
+        <v>2322</v>
       </c>
       <c r="N15" s="31" t="inlineStr">
         <is>
@@ -3391,34 +3391,34 @@
         <v>727</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>37.9</v>
+        <v>30.8</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>275</v>
+        <v>224</v>
       </c>
       <c r="F16" s="30" t="n">
-        <v>38.2</v>
+        <v>39.4</v>
       </c>
       <c r="G16" s="30" t="n">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="H16" s="30" t="n">
-        <v>23.2</v>
+        <v>13.5</v>
       </c>
       <c r="I16" s="30" t="n">
-        <v>169</v>
+        <v>98</v>
       </c>
       <c r="J16" s="30" t="n">
-        <v>0.7</v>
+        <v>16.3</v>
       </c>
       <c r="K16" s="30" t="n">
-        <v>5</v>
+        <v>119</v>
       </c>
       <c r="L16" s="30" t="n">
-        <v>62.1</v>
+        <v>69.2</v>
       </c>
       <c r="M16" s="30" t="n">
-        <v>452</v>
+        <v>503</v>
       </c>
       <c r="N16" s="31" t="inlineStr">
         <is>
@@ -3569,38 +3569,38 @@
         <v>2160</v>
       </c>
       <c r="D17" s="30" t="n">
-        <v>38.9</v>
+        <v>34.6</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>840</v>
+        <v>748</v>
       </c>
       <c r="F17" s="30" t="n">
-        <v>41.1</v>
+        <v>33.2</v>
       </c>
       <c r="G17" s="30" t="n">
-        <v>889</v>
+        <v>717</v>
       </c>
       <c r="H17" s="30" t="n">
-        <v>19.7</v>
+        <v>13.2</v>
       </c>
       <c r="I17" s="30" t="n">
-        <v>425</v>
+        <v>285</v>
       </c>
       <c r="J17" s="30" t="n">
-        <v>0.3</v>
+        <v>19</v>
       </c>
       <c r="K17" s="30" t="n">
-        <v>7</v>
+        <v>410</v>
       </c>
       <c r="L17" s="30" t="n">
-        <v>61.1</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="M17" s="30" t="n">
-        <v>1321</v>
+        <v>1413</v>
       </c>
       <c r="N17" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O17" s="32" t="n">
@@ -3747,34 +3747,34 @@
         <v>12099</v>
       </c>
       <c r="D18" s="30" t="n">
-        <v>37.4</v>
+        <v>37.2</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>4523</v>
+        <v>4496</v>
       </c>
       <c r="F18" s="30" t="n">
-        <v>55.2</v>
+        <v>51.2</v>
       </c>
       <c r="G18" s="30" t="n">
-        <v>6677</v>
+        <v>6199</v>
       </c>
       <c r="H18" s="30" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I18" s="30" t="n">
-        <v>822</v>
+        <v>734</v>
       </c>
       <c r="J18" s="30" t="n">
-        <v>0.6</v>
+        <v>5.5</v>
       </c>
       <c r="K18" s="30" t="n">
-        <v>76</v>
+        <v>669</v>
       </c>
       <c r="L18" s="30" t="n">
-        <v>62.6</v>
+        <v>62.8</v>
       </c>
       <c r="M18" s="30" t="n">
-        <v>7575</v>
+        <v>7602</v>
       </c>
       <c r="N18" s="31" t="inlineStr">
         <is>
@@ -3925,34 +3925,34 @@
         <v>5108</v>
       </c>
       <c r="D19" s="30" t="n">
-        <v>54.6</v>
+        <v>53.5</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>2789</v>
+        <v>2733</v>
       </c>
       <c r="F19" s="30" t="n">
-        <v>32.6</v>
+        <v>30.3</v>
       </c>
       <c r="G19" s="30" t="n">
-        <v>1665</v>
+        <v>1547</v>
       </c>
       <c r="H19" s="30" t="n">
-        <v>12.8</v>
+        <v>4.3</v>
       </c>
       <c r="I19" s="30" t="n">
-        <v>653</v>
+        <v>219</v>
       </c>
       <c r="J19" s="30" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="K19" s="30" t="n">
-        <v>0</v>
+        <v>609</v>
       </c>
       <c r="L19" s="30" t="n">
-        <v>45.4</v>
+        <v>46.5</v>
       </c>
       <c r="M19" s="30" t="n">
-        <v>2319</v>
+        <v>2375</v>
       </c>
       <c r="N19" s="31" t="inlineStr">
         <is>
@@ -4117,34 +4117,34 @@
         <v>4659</v>
       </c>
       <c r="D20" s="30" t="n">
-        <v>57.3</v>
+        <v>54.1</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>2671</v>
+        <v>2522</v>
       </c>
       <c r="F20" s="30" t="n">
-        <v>36.9</v>
+        <v>37</v>
       </c>
       <c r="G20" s="30" t="n">
-        <v>1721</v>
+        <v>1724</v>
       </c>
       <c r="H20" s="30" t="n">
-        <v>5.7</v>
+        <v>3.6</v>
       </c>
       <c r="I20" s="30" t="n">
-        <v>265</v>
+        <v>167</v>
       </c>
       <c r="J20" s="30" t="n">
-        <v>0.1</v>
+        <v>5.3</v>
       </c>
       <c r="K20" s="30" t="n">
-        <v>3</v>
+        <v>246</v>
       </c>
       <c r="L20" s="30" t="n">
-        <v>42.7</v>
+        <v>45.9</v>
       </c>
       <c r="M20" s="30" t="n">
-        <v>1988</v>
+        <v>2137</v>
       </c>
       <c r="N20" s="31" t="inlineStr">
         <is>
@@ -4295,34 +4295,34 @@
         <v>5046</v>
       </c>
       <c r="D21" s="30" t="n">
-        <v>51.9</v>
+        <v>50.9</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>2618</v>
+        <v>2567</v>
       </c>
       <c r="F21" s="30" t="n">
-        <v>29</v>
+        <v>30.3</v>
       </c>
       <c r="G21" s="30" t="n">
-        <v>1464</v>
+        <v>1529</v>
       </c>
       <c r="H21" s="30" t="n">
-        <v>18.7</v>
+        <v>3.5</v>
       </c>
       <c r="I21" s="30" t="n">
-        <v>942</v>
+        <v>178</v>
       </c>
       <c r="J21" s="30" t="n">
-        <v>0.4</v>
+        <v>15.3</v>
       </c>
       <c r="K21" s="30" t="n">
-        <v>22</v>
+        <v>772</v>
       </c>
       <c r="L21" s="30" t="n">
-        <v>48.1</v>
+        <v>49.1</v>
       </c>
       <c r="M21" s="30" t="n">
-        <v>2428</v>
+        <v>2479</v>
       </c>
       <c r="N21" s="31" t="inlineStr">
         <is>
@@ -4473,34 +4473,34 @@
         <v>20269</v>
       </c>
       <c r="D22" s="30" t="n">
-        <v>69.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>14132</v>
+        <v>14103</v>
       </c>
       <c r="F22" s="30" t="n">
-        <v>19.5</v>
+        <v>20</v>
       </c>
       <c r="G22" s="30" t="n">
-        <v>3944</v>
+        <v>4058</v>
       </c>
       <c r="H22" s="30" t="n">
-        <v>9.800000000000001</v>
+        <v>1.8</v>
       </c>
       <c r="I22" s="30" t="n">
-        <v>1990</v>
+        <v>372</v>
       </c>
       <c r="J22" s="30" t="n">
-        <v>1</v>
+        <v>8.6</v>
       </c>
       <c r="K22" s="30" t="n">
-        <v>204</v>
+        <v>1737</v>
       </c>
       <c r="L22" s="30" t="n">
-        <v>30.3</v>
+        <v>30.4</v>
       </c>
       <c r="M22" s="30" t="n">
-        <v>6137</v>
+        <v>6167</v>
       </c>
       <c r="N22" s="31" t="inlineStr">
         <is>
@@ -4651,38 +4651,38 @@
         <v>10200</v>
       </c>
       <c r="D23" s="30" t="n">
-        <v>56.3</v>
+        <v>53.3</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>5745</v>
+        <v>5435</v>
       </c>
       <c r="F23" s="30" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="G23" s="30" t="n">
-        <v>2496</v>
+        <v>2519</v>
       </c>
       <c r="H23" s="30" t="n">
-        <v>18.9</v>
+        <v>5.4</v>
       </c>
       <c r="I23" s="30" t="n">
-        <v>1923</v>
+        <v>554</v>
       </c>
       <c r="J23" s="30" t="n">
-        <v>0.4</v>
+        <v>16.6</v>
       </c>
       <c r="K23" s="30" t="n">
-        <v>36</v>
+        <v>1693</v>
       </c>
       <c r="L23" s="30" t="n">
-        <v>43.7</v>
+        <v>46.7</v>
       </c>
       <c r="M23" s="30" t="n">
-        <v>4455</v>
+        <v>4765</v>
       </c>
       <c r="N23" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O23" s="32" t="n">
@@ -4829,38 +4829,38 @@
         <v>9179</v>
       </c>
       <c r="D24" s="30" t="n">
-        <v>28.1</v>
+        <v>27.9</v>
       </c>
       <c r="E24" s="30" t="n">
-        <v>2575</v>
+        <v>2558</v>
       </c>
       <c r="F24" s="30" t="n">
-        <v>42.7</v>
+        <v>43.2</v>
       </c>
       <c r="G24" s="30" t="n">
-        <v>3919</v>
+        <v>3962</v>
       </c>
       <c r="H24" s="30" t="n">
-        <v>29.1</v>
+        <v>3.8</v>
       </c>
       <c r="I24" s="30" t="n">
-        <v>2668</v>
+        <v>345</v>
       </c>
       <c r="J24" s="30" t="n">
-        <v>0.2</v>
+        <v>25.2</v>
       </c>
       <c r="K24" s="30" t="n">
-        <v>17</v>
+        <v>2313</v>
       </c>
       <c r="L24" s="30" t="n">
-        <v>71.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="M24" s="30" t="n">
-        <v>6604</v>
+        <v>6621</v>
       </c>
       <c r="N24" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O24" s="32" t="n">
@@ -5007,34 +5007,34 @@
         <v>1812</v>
       </c>
       <c r="D25" s="30" t="n">
-        <v>38.5</v>
+        <v>37.9</v>
       </c>
       <c r="E25" s="30" t="n">
-        <v>698</v>
+        <v>687</v>
       </c>
       <c r="F25" s="30" t="n">
-        <v>39.1</v>
+        <v>39.6</v>
       </c>
       <c r="G25" s="30" t="n">
-        <v>709</v>
+        <v>718</v>
       </c>
       <c r="H25" s="30" t="n">
-        <v>22.1</v>
+        <v>4.3</v>
       </c>
       <c r="I25" s="30" t="n">
-        <v>400</v>
+        <v>78</v>
       </c>
       <c r="J25" s="30" t="n">
-        <v>0.3</v>
+        <v>18.2</v>
       </c>
       <c r="K25" s="30" t="n">
-        <v>5</v>
+        <v>329</v>
       </c>
       <c r="L25" s="30" t="n">
-        <v>61.5</v>
+        <v>62.1</v>
       </c>
       <c r="M25" s="30" t="n">
-        <v>1114</v>
+        <v>1124</v>
       </c>
       <c r="N25" s="31" t="inlineStr">
         <is>
@@ -5185,38 +5185,38 @@
         <v>4386</v>
       </c>
       <c r="D26" s="30" t="n">
-        <v>45.1</v>
+        <v>40.9</v>
       </c>
       <c r="E26" s="30" t="n">
-        <v>1979</v>
+        <v>1793</v>
       </c>
       <c r="F26" s="30" t="n">
-        <v>38.6</v>
+        <v>35.4</v>
       </c>
       <c r="G26" s="30" t="n">
-        <v>1694</v>
+        <v>1553</v>
       </c>
       <c r="H26" s="30" t="n">
-        <v>16.2</v>
+        <v>10.6</v>
       </c>
       <c r="I26" s="30" t="n">
-        <v>713</v>
+        <v>466</v>
       </c>
       <c r="J26" s="30" t="n">
-        <v>0</v>
+        <v>13.1</v>
       </c>
       <c r="K26" s="30" t="n">
-        <v>0</v>
+        <v>574</v>
       </c>
       <c r="L26" s="30" t="n">
-        <v>54.9</v>
+        <v>59.1</v>
       </c>
       <c r="M26" s="30" t="n">
-        <v>2407</v>
+        <v>2593</v>
       </c>
       <c r="N26" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O26" s="32" t="n">
@@ -5363,34 +5363,34 @@
         <v>297</v>
       </c>
       <c r="D27" s="30" t="n">
-        <v>62.2</v>
+        <v>61.5</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F27" s="30" t="n">
-        <v>26.4</v>
+        <v>25.2</v>
       </c>
       <c r="G27" s="30" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H27" s="30" t="n">
-        <v>11.4</v>
+        <v>3</v>
       </c>
       <c r="I27" s="30" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="J27" s="30" t="n">
-        <v>0</v>
+        <v>10.2</v>
       </c>
       <c r="K27" s="30" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L27" s="30" t="n">
-        <v>37.8</v>
+        <v>38.5</v>
       </c>
       <c r="M27" s="30" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N27" s="31" t="inlineStr">
         <is>
@@ -5541,38 +5541,38 @@
         <v>446</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>54.7</v>
+        <v>53.1</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="F28" s="30" t="n">
-        <v>28.6</v>
+        <v>24.3</v>
       </c>
       <c r="G28" s="30" t="n">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="H28" s="30" t="n">
-        <v>15.6</v>
+        <v>10.3</v>
       </c>
       <c r="I28" s="30" t="n">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="J28" s="30" t="n">
-        <v>1.1</v>
+        <v>12.3</v>
       </c>
       <c r="K28" s="30" t="n">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="L28" s="30" t="n">
-        <v>45.3</v>
+        <v>46.9</v>
       </c>
       <c r="M28" s="30" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="N28" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O28" s="32" t="n">
@@ -5725,22 +5725,22 @@
         <v>117</v>
       </c>
       <c r="F29" s="30" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G29" s="30" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="H29" s="30" t="n">
-        <v>11.7</v>
+        <v>8.5</v>
       </c>
       <c r="I29" s="30" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="J29" s="30" t="n">
-        <v>1.5</v>
+        <v>8.6</v>
       </c>
       <c r="K29" s="30" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="L29" s="30" t="n">
         <v>54.1</v>
@@ -5897,38 +5897,38 @@
         <v>1288</v>
       </c>
       <c r="D30" s="30" t="n">
-        <v>42</v>
+        <v>38.3</v>
       </c>
       <c r="E30" s="30" t="n">
-        <v>540</v>
+        <v>493</v>
       </c>
       <c r="F30" s="30" t="n">
-        <v>45.2</v>
+        <v>41.7</v>
       </c>
       <c r="G30" s="30" t="n">
-        <v>583</v>
+        <v>537</v>
       </c>
       <c r="H30" s="30" t="n">
-        <v>12.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I30" s="30" t="n">
-        <v>157</v>
+        <v>113</v>
       </c>
       <c r="J30" s="30" t="n">
-        <v>0.6</v>
+        <v>11.3</v>
       </c>
       <c r="K30" s="30" t="n">
-        <v>8</v>
+        <v>146</v>
       </c>
       <c r="L30" s="30" t="n">
-        <v>58</v>
+        <v>61.7</v>
       </c>
       <c r="M30" s="30" t="n">
-        <v>747</v>
+        <v>795</v>
       </c>
       <c r="N30" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O30" s="32" t="n">
@@ -6075,34 +6075,34 @@
         <v>1279</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>70.59999999999999</v>
+        <v>70</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>903</v>
+        <v>896</v>
       </c>
       <c r="F31" s="30" t="n">
-        <v>23.9</v>
+        <v>23.6</v>
       </c>
       <c r="G31" s="30" t="n">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="H31" s="30" t="n">
-        <v>5.5</v>
+        <v>2.2</v>
       </c>
       <c r="I31" s="30" t="n">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="J31" s="30" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="K31" s="30" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="L31" s="30" t="n">
-        <v>29.4</v>
+        <v>30</v>
       </c>
       <c r="M31" s="30" t="n">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="N31" s="31" t="inlineStr">
         <is>
@@ -6259,22 +6259,22 @@
         <v>2877</v>
       </c>
       <c r="F32" s="30" t="n">
-        <v>22.3</v>
+        <v>22.7</v>
       </c>
       <c r="G32" s="30" t="n">
-        <v>1125</v>
+        <v>1148</v>
       </c>
       <c r="H32" s="30" t="n">
-        <v>20.1</v>
+        <v>1.1</v>
       </c>
       <c r="I32" s="30" t="n">
-        <v>1016</v>
+        <v>56</v>
       </c>
       <c r="J32" s="30" t="n">
-        <v>0.7</v>
+        <v>19.2</v>
       </c>
       <c r="K32" s="30" t="n">
-        <v>35</v>
+        <v>972</v>
       </c>
       <c r="L32" s="30" t="n">
         <v>43.1</v>
@@ -6431,38 +6431,38 @@
         <v>1368</v>
       </c>
       <c r="D33" s="30" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="F33" s="30" t="n">
-        <v>32.4</v>
+        <v>30.6</v>
       </c>
       <c r="G33" s="30" t="n">
-        <v>443</v>
+        <v>418</v>
       </c>
       <c r="H33" s="30" t="n">
-        <v>23.9</v>
+        <v>5.4</v>
       </c>
       <c r="I33" s="30" t="n">
-        <v>327</v>
+        <v>73</v>
       </c>
       <c r="J33" s="30" t="n">
-        <v>0.7</v>
+        <v>21.3</v>
       </c>
       <c r="K33" s="30" t="n">
-        <v>9</v>
+        <v>292</v>
       </c>
       <c r="L33" s="30" t="n">
-        <v>57</v>
+        <v>57.2</v>
       </c>
       <c r="M33" s="30" t="n">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="N33" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O33" s="32" t="n">
@@ -6609,38 +6609,38 @@
         <v>3024</v>
       </c>
       <c r="D34" s="30" t="n">
-        <v>20.1</v>
+        <v>18.1</v>
       </c>
       <c r="E34" s="30" t="n">
-        <v>608</v>
+        <v>546</v>
       </c>
       <c r="F34" s="30" t="n">
-        <v>45.6</v>
+        <v>28.5</v>
       </c>
       <c r="G34" s="30" t="n">
-        <v>1379</v>
+        <v>862</v>
       </c>
       <c r="H34" s="30" t="n">
-        <v>33.9</v>
+        <v>28.4</v>
       </c>
       <c r="I34" s="30" t="n">
-        <v>1026</v>
+        <v>858</v>
       </c>
       <c r="J34" s="30" t="n">
-        <v>0.4</v>
+        <v>25</v>
       </c>
       <c r="K34" s="30" t="n">
-        <v>11</v>
+        <v>757</v>
       </c>
       <c r="L34" s="30" t="n">
-        <v>79.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="M34" s="30" t="n">
-        <v>2416</v>
+        <v>2478</v>
       </c>
       <c r="N34" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O34" s="32" t="n">
@@ -6787,34 +6787,34 @@
         <v>10362</v>
       </c>
       <c r="D35" s="30" t="n">
-        <v>62.9</v>
+        <v>61.4</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>6517</v>
+        <v>6361</v>
       </c>
       <c r="F35" s="30" t="n">
-        <v>23.3</v>
+        <v>24.1</v>
       </c>
       <c r="G35" s="30" t="n">
-        <v>2416</v>
+        <v>2502</v>
       </c>
       <c r="H35" s="30" t="n">
-        <v>13.7</v>
+        <v>2.7</v>
       </c>
       <c r="I35" s="30" t="n">
-        <v>1422</v>
+        <v>281</v>
       </c>
       <c r="J35" s="30" t="n">
-        <v>0.1</v>
+        <v>11.8</v>
       </c>
       <c r="K35" s="30" t="n">
-        <v>8</v>
+        <v>1218</v>
       </c>
       <c r="L35" s="30" t="n">
-        <v>37.1</v>
+        <v>38.6</v>
       </c>
       <c r="M35" s="30" t="n">
-        <v>3846</v>
+        <v>4002</v>
       </c>
       <c r="N35" s="31" t="inlineStr">
         <is>
@@ -6965,34 +6965,34 @@
         <v>2077</v>
       </c>
       <c r="D36" s="30" t="n">
-        <v>73.5</v>
+        <v>73.3</v>
       </c>
       <c r="E36" s="30" t="n">
-        <v>1527</v>
+        <v>1522</v>
       </c>
       <c r="F36" s="30" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
       <c r="G36" s="30" t="n">
-        <v>401</v>
+        <v>385</v>
       </c>
       <c r="H36" s="30" t="n">
-        <v>7.2</v>
+        <v>1.2</v>
       </c>
       <c r="I36" s="30" t="n">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="J36" s="30" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K36" s="30" t="n">
-        <v>1</v>
+        <v>145</v>
       </c>
       <c r="L36" s="30" t="n">
-        <v>26.5</v>
+        <v>26.7</v>
       </c>
       <c r="M36" s="30" t="n">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="N36" s="31" t="inlineStr">
         <is>
@@ -7321,34 +7321,34 @@
         <v>21627</v>
       </c>
       <c r="D38" s="30" t="n">
-        <v>65.7</v>
+        <v>65.2</v>
       </c>
       <c r="E38" s="30" t="n">
-        <v>14213</v>
+        <v>14103</v>
       </c>
       <c r="F38" s="30" t="n">
-        <v>25</v>
+        <v>20.6</v>
       </c>
       <c r="G38" s="30" t="n">
-        <v>5413</v>
+        <v>4461</v>
       </c>
       <c r="H38" s="30" t="n">
-        <v>9.1</v>
+        <v>5.5</v>
       </c>
       <c r="I38" s="30" t="n">
-        <v>1960</v>
+        <v>1198</v>
       </c>
       <c r="J38" s="30" t="n">
-        <v>0.2</v>
+        <v>8.6</v>
       </c>
       <c r="K38" s="30" t="n">
-        <v>41</v>
+        <v>1865</v>
       </c>
       <c r="L38" s="30" t="n">
-        <v>34.3</v>
+        <v>34.8</v>
       </c>
       <c r="M38" s="30" t="n">
-        <v>7414</v>
+        <v>7524</v>
       </c>
       <c r="N38" s="31" t="inlineStr">
         <is>
@@ -7499,38 +7499,38 @@
         <v>4670</v>
       </c>
       <c r="D39" s="30" t="n">
-        <v>35.7</v>
+        <v>34.1</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>1666</v>
+        <v>1595</v>
       </c>
       <c r="F39" s="30" t="n">
-        <v>29.5</v>
+        <v>22</v>
       </c>
       <c r="G39" s="30" t="n">
-        <v>1378</v>
+        <v>1029</v>
       </c>
       <c r="H39" s="30" t="n">
-        <v>34.3</v>
+        <v>17.8</v>
       </c>
       <c r="I39" s="30" t="n">
-        <v>1603</v>
+        <v>832</v>
       </c>
       <c r="J39" s="30" t="n">
-        <v>0.5</v>
+        <v>26</v>
       </c>
       <c r="K39" s="30" t="n">
-        <v>24</v>
+        <v>1215</v>
       </c>
       <c r="L39" s="30" t="n">
-        <v>64.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="M39" s="30" t="n">
-        <v>3005</v>
+        <v>3076</v>
       </c>
       <c r="N39" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O39" s="32" t="n">
@@ -7677,34 +7677,34 @@
         <v>12568</v>
       </c>
       <c r="D40" s="30" t="n">
-        <v>75.90000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="E40" s="30" t="n">
-        <v>9542</v>
+        <v>9241</v>
       </c>
       <c r="F40" s="30" t="n">
-        <v>13.9</v>
+        <v>16.3</v>
       </c>
       <c r="G40" s="30" t="n">
-        <v>1746</v>
+        <v>2055</v>
       </c>
       <c r="H40" s="30" t="n">
-        <v>9.4</v>
+        <v>1.9</v>
       </c>
       <c r="I40" s="30" t="n">
-        <v>1176</v>
+        <v>237</v>
       </c>
       <c r="J40" s="30" t="n">
-        <v>0.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K40" s="30" t="n">
-        <v>104</v>
+        <v>1035</v>
       </c>
       <c r="L40" s="30" t="n">
-        <v>24.1</v>
+        <v>26.5</v>
       </c>
       <c r="M40" s="30" t="n">
-        <v>3026</v>
+        <v>3327</v>
       </c>
       <c r="N40" s="31" t="inlineStr">
         <is>
@@ -7855,34 +7855,34 @@
         <v>6763</v>
       </c>
       <c r="D41" s="30" t="n">
-        <v>68.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="E41" s="30" t="n">
-        <v>4628</v>
+        <v>4589</v>
       </c>
       <c r="F41" s="30" t="n">
-        <v>24.6</v>
+        <v>25.6</v>
       </c>
       <c r="G41" s="30" t="n">
-        <v>1663</v>
+        <v>1733</v>
       </c>
       <c r="H41" s="30" t="n">
-        <v>6.6</v>
+        <v>0.8</v>
       </c>
       <c r="I41" s="30" t="n">
-        <v>449</v>
+        <v>52</v>
       </c>
       <c r="J41" s="30" t="n">
-        <v>0.4</v>
+        <v>5.7</v>
       </c>
       <c r="K41" s="30" t="n">
-        <v>24</v>
+        <v>389</v>
       </c>
       <c r="L41" s="30" t="n">
-        <v>31.6</v>
+        <v>32.2</v>
       </c>
       <c r="M41" s="30" t="n">
-        <v>2135</v>
+        <v>2174</v>
       </c>
       <c r="N41" s="31" t="inlineStr">
         <is>
@@ -8033,34 +8033,34 @@
         <v>985</v>
       </c>
       <c r="D42" s="30" t="n">
-        <v>58.4</v>
+        <v>58.2</v>
       </c>
       <c r="E42" s="30" t="n">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="F42" s="30" t="n">
-        <v>37.6</v>
+        <v>37.9</v>
       </c>
       <c r="G42" s="30" t="n">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="H42" s="30" t="n">
-        <v>4</v>
+        <v>0.6</v>
       </c>
       <c r="I42" s="30" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="J42" s="30" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="K42" s="30" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L42" s="30" t="n">
-        <v>41.6</v>
+        <v>41.8</v>
       </c>
       <c r="M42" s="30" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="N42" s="31" t="inlineStr">
         <is>
@@ -8211,34 +8211,34 @@
         <v>13517</v>
       </c>
       <c r="D43" s="30" t="n">
-        <v>62.6</v>
+        <v>62.3</v>
       </c>
       <c r="E43" s="30" t="n">
-        <v>8456</v>
+        <v>8418</v>
       </c>
       <c r="F43" s="30" t="n">
-        <v>18.2</v>
+        <v>20.8</v>
       </c>
       <c r="G43" s="30" t="n">
-        <v>2466</v>
+        <v>2815</v>
       </c>
       <c r="H43" s="30" t="n">
-        <v>19.1</v>
+        <v>0.3</v>
       </c>
       <c r="I43" s="30" t="n">
-        <v>2576</v>
+        <v>42</v>
       </c>
       <c r="J43" s="30" t="n">
-        <v>0.1</v>
+        <v>16.6</v>
       </c>
       <c r="K43" s="30" t="n">
-        <v>18</v>
+        <v>2242</v>
       </c>
       <c r="L43" s="30" t="n">
-        <v>37.4</v>
+        <v>37.7</v>
       </c>
       <c r="M43" s="30" t="n">
-        <v>5061</v>
+        <v>5099</v>
       </c>
       <c r="N43" s="31" t="inlineStr">
         <is>
@@ -8389,34 +8389,34 @@
         <v>1387</v>
       </c>
       <c r="D44" s="30" t="n">
-        <v>40.4</v>
+        <v>38.3</v>
       </c>
       <c r="E44" s="30" t="n">
-        <v>561</v>
+        <v>531</v>
       </c>
       <c r="F44" s="30" t="n">
-        <v>47</v>
+        <v>47.2</v>
       </c>
       <c r="G44" s="30" t="n">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="H44" s="30" t="n">
-        <v>12.3</v>
+        <v>3.7</v>
       </c>
       <c r="I44" s="30" t="n">
-        <v>170</v>
+        <v>52</v>
       </c>
       <c r="J44" s="30" t="n">
-        <v>0.3</v>
+        <v>10.8</v>
       </c>
       <c r="K44" s="30" t="n">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="L44" s="30" t="n">
-        <v>59.6</v>
+        <v>61.7</v>
       </c>
       <c r="M44" s="30" t="n">
-        <v>826</v>
+        <v>857</v>
       </c>
       <c r="N44" s="31" t="inlineStr">
         <is>
@@ -8567,38 +8567,38 @@
         <v>82</v>
       </c>
       <c r="D45" s="30" t="n">
-        <v>38.8</v>
+        <v>36.3</v>
       </c>
       <c r="E45" s="30" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F45" s="30" t="n">
-        <v>41.6</v>
+        <v>37.3</v>
       </c>
       <c r="G45" s="30" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H45" s="30" t="n">
-        <v>18.7</v>
+        <v>9.9</v>
       </c>
       <c r="I45" s="30" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="J45" s="30" t="n">
-        <v>0.9</v>
+        <v>16.5</v>
       </c>
       <c r="K45" s="30" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="L45" s="30" t="n">
-        <v>61.2</v>
+        <v>63.7</v>
       </c>
       <c r="M45" s="30" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N45" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O45" s="32" t="n">
@@ -8751,22 +8751,22 @@
         <v>879</v>
       </c>
       <c r="F46" s="30" t="n">
-        <v>14.5</v>
+        <v>12.1</v>
       </c>
       <c r="G46" s="30" t="n">
-        <v>188</v>
+        <v>156</v>
       </c>
       <c r="H46" s="30" t="n">
-        <v>16.9</v>
+        <v>3.4</v>
       </c>
       <c r="I46" s="30" t="n">
-        <v>219</v>
+        <v>44</v>
       </c>
       <c r="J46" s="30" t="n">
-        <v>0.6</v>
+        <v>16.6</v>
       </c>
       <c r="K46" s="30" t="n">
-        <v>8</v>
+        <v>215</v>
       </c>
       <c r="L46" s="30" t="n">
         <v>32.1</v>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="N46" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O46" s="32" t="n">
@@ -8943,38 +8943,38 @@
         <v>4404</v>
       </c>
       <c r="D47" s="30" t="n">
-        <v>38.6</v>
+        <v>35.8</v>
       </c>
       <c r="E47" s="30" t="n">
-        <v>1701</v>
+        <v>1575</v>
       </c>
       <c r="F47" s="30" t="n">
-        <v>29.2</v>
+        <v>28.1</v>
       </c>
       <c r="G47" s="30" t="n">
-        <v>1286</v>
+        <v>1237</v>
       </c>
       <c r="H47" s="30" t="n">
-        <v>30.9</v>
+        <v>6.7</v>
       </c>
       <c r="I47" s="30" t="n">
-        <v>1362</v>
+        <v>293</v>
       </c>
       <c r="J47" s="30" t="n">
-        <v>1.2</v>
+        <v>29.5</v>
       </c>
       <c r="K47" s="30" t="n">
-        <v>55</v>
+        <v>1299</v>
       </c>
       <c r="L47" s="30" t="n">
-        <v>61.4</v>
+        <v>64.2</v>
       </c>
       <c r="M47" s="30" t="n">
-        <v>2703</v>
+        <v>2829</v>
       </c>
       <c r="N47" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O47" s="32" t="n">
@@ -9295,22 +9295,22 @@
         <v>3024</v>
       </c>
       <c r="F49" s="30" t="n">
-        <v>23.5</v>
+        <v>19.1</v>
       </c>
       <c r="G49" s="30" t="n">
-        <v>1024</v>
+        <v>832</v>
       </c>
       <c r="H49" s="30" t="n">
-        <v>6.8</v>
+        <v>5.4</v>
       </c>
       <c r="I49" s="30" t="n">
-        <v>295</v>
+        <v>237</v>
       </c>
       <c r="J49" s="30" t="n">
-        <v>0.4</v>
+        <v>6.1</v>
       </c>
       <c r="K49" s="30" t="n">
-        <v>15</v>
+        <v>266</v>
       </c>
       <c r="L49" s="30" t="n">
         <v>30.6</v>
@@ -9467,34 +9467,34 @@
         <v>11294</v>
       </c>
       <c r="D50" s="30" t="n">
-        <v>52.1</v>
+        <v>50</v>
       </c>
       <c r="E50" s="30" t="n">
-        <v>5884</v>
+        <v>5647</v>
       </c>
       <c r="F50" s="30" t="n">
-        <v>24.1</v>
+        <v>29.2</v>
       </c>
       <c r="G50" s="30" t="n">
-        <v>2727</v>
+        <v>3301</v>
       </c>
       <c r="H50" s="30" t="n">
-        <v>22.3</v>
+        <v>1</v>
       </c>
       <c r="I50" s="30" t="n">
-        <v>2521</v>
+        <v>108</v>
       </c>
       <c r="J50" s="30" t="n">
-        <v>1.4</v>
+        <v>19.8</v>
       </c>
       <c r="K50" s="30" t="n">
-        <v>162</v>
+        <v>2239</v>
       </c>
       <c r="L50" s="30" t="n">
-        <v>47.9</v>
+        <v>50</v>
       </c>
       <c r="M50" s="30" t="n">
-        <v>5411</v>
+        <v>5647</v>
       </c>
       <c r="N50" s="31" t="inlineStr">
         <is>
@@ -9829,22 +9829,22 @@
         <v>3400</v>
       </c>
       <c r="F52" s="30" t="n">
-        <v>33.4</v>
+        <v>31.4</v>
       </c>
       <c r="G52" s="30" t="n">
-        <v>2347</v>
+        <v>2205</v>
       </c>
       <c r="H52" s="30" t="n">
-        <v>17.8</v>
+        <v>5.7</v>
       </c>
       <c r="I52" s="30" t="n">
-        <v>1250</v>
+        <v>400</v>
       </c>
       <c r="J52" s="30" t="n">
-        <v>0.3</v>
+        <v>14.4</v>
       </c>
       <c r="K52" s="30" t="n">
-        <v>23</v>
+        <v>1014</v>
       </c>
       <c r="L52" s="30" t="n">
         <v>51.6</v>
@@ -9854,7 +9854,7 @@
       </c>
       <c r="N52" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O52" s="32" t="n">
@@ -10001,38 +10001,38 @@
         <v>713</v>
       </c>
       <c r="D53" s="30" t="n">
-        <v>26.4</v>
+        <v>24.4</v>
       </c>
       <c r="E53" s="30" t="n">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="F53" s="30" t="n">
-        <v>39</v>
+        <v>41.3</v>
       </c>
       <c r="G53" s="30" t="n">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="H53" s="30" t="n">
-        <v>34</v>
+        <v>0.6</v>
       </c>
       <c r="I53" s="30" t="n">
-        <v>242</v>
+        <v>4</v>
       </c>
       <c r="J53" s="30" t="n">
-        <v>0.6</v>
+        <v>33.6</v>
       </c>
       <c r="K53" s="30" t="n">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="L53" s="30" t="n">
-        <v>73.59999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="M53" s="30" t="n">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="N53" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O53" s="32" t="n">
@@ -10199,34 +10199,34 @@
         <v>1532</v>
       </c>
       <c r="D54" s="30" t="n">
-        <v>65.90000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="E54" s="30" t="n">
-        <v>1010</v>
+        <v>1006</v>
       </c>
       <c r="F54" s="30" t="n">
-        <v>21.6</v>
+        <v>20.2</v>
       </c>
       <c r="G54" s="30" t="n">
-        <v>331</v>
+        <v>309</v>
       </c>
       <c r="H54" s="30" t="n">
-        <v>12.5</v>
+        <v>2.8</v>
       </c>
       <c r="I54" s="30" t="n">
-        <v>191</v>
+        <v>43</v>
       </c>
       <c r="J54" s="30" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="K54" s="30" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="L54" s="30" t="n">
-        <v>34.1</v>
+        <v>34.3</v>
       </c>
       <c r="M54" s="30" t="n">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="N54" s="31" t="inlineStr">
         <is>
@@ -10555,38 +10555,38 @@
         <v>945</v>
       </c>
       <c r="D56" s="30" t="n">
-        <v>31.6</v>
+        <v>30.6</v>
       </c>
       <c r="E56" s="30" t="n">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="F56" s="30" t="n">
-        <v>34.8</v>
+        <v>31.3</v>
       </c>
       <c r="G56" s="30" t="n">
-        <v>329</v>
+        <v>296</v>
       </c>
       <c r="H56" s="30" t="n">
-        <v>33.2</v>
+        <v>7.4</v>
       </c>
       <c r="I56" s="30" t="n">
-        <v>314</v>
+        <v>70</v>
       </c>
       <c r="J56" s="30" t="n">
-        <v>0.3</v>
+        <v>30.7</v>
       </c>
       <c r="K56" s="30" t="n">
-        <v>3</v>
+        <v>290</v>
       </c>
       <c r="L56" s="30" t="n">
-        <v>68.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="M56" s="30" t="n">
-        <v>646</v>
+        <v>656</v>
       </c>
       <c r="N56" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O56" s="32" t="n">
@@ -10733,34 +10733,34 @@
         <v>3722</v>
       </c>
       <c r="D57" s="30" t="n">
-        <v>63.5</v>
+        <v>63.1</v>
       </c>
       <c r="E57" s="30" t="n">
-        <v>2363</v>
+        <v>2349</v>
       </c>
       <c r="F57" s="30" t="n">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="G57" s="30" t="n">
-        <v>780</v>
+        <v>774</v>
       </c>
       <c r="H57" s="30" t="n">
-        <v>15.1</v>
+        <v>3</v>
       </c>
       <c r="I57" s="30" t="n">
-        <v>562</v>
+        <v>111</v>
       </c>
       <c r="J57" s="30" t="n">
-        <v>0.4</v>
+        <v>13.1</v>
       </c>
       <c r="K57" s="30" t="n">
-        <v>17</v>
+        <v>487</v>
       </c>
       <c r="L57" s="30" t="n">
-        <v>36.5</v>
+        <v>36.9</v>
       </c>
       <c r="M57" s="30" t="n">
-        <v>1358</v>
+        <v>1372</v>
       </c>
       <c r="N57" s="31" t="inlineStr">
         <is>
@@ -10911,34 +10911,34 @@
         <v>7021</v>
       </c>
       <c r="D58" s="30" t="n">
-        <v>58</v>
+        <v>56.5</v>
       </c>
       <c r="E58" s="30" t="n">
-        <v>4072</v>
+        <v>3969</v>
       </c>
       <c r="F58" s="30" t="n">
-        <v>29.8</v>
+        <v>28.8</v>
       </c>
       <c r="G58" s="30" t="n">
-        <v>2095</v>
+        <v>2024</v>
       </c>
       <c r="H58" s="30" t="n">
-        <v>11.9</v>
+        <v>5.6</v>
       </c>
       <c r="I58" s="30" t="n">
-        <v>839</v>
+        <v>395</v>
       </c>
       <c r="J58" s="30" t="n">
-        <v>0.2</v>
+        <v>9</v>
       </c>
       <c r="K58" s="30" t="n">
-        <v>15</v>
+        <v>633</v>
       </c>
       <c r="L58" s="30" t="n">
-        <v>42</v>
+        <v>43.5</v>
       </c>
       <c r="M58" s="30" t="n">
-        <v>2949</v>
+        <v>3052</v>
       </c>
       <c r="N58" s="31" t="inlineStr">
         <is>
@@ -11095,22 +11095,22 @@
         <v>2787</v>
       </c>
       <c r="F59" s="30" t="n">
-        <v>35.1</v>
+        <v>32.9</v>
       </c>
       <c r="G59" s="30" t="n">
-        <v>1817</v>
+        <v>1701</v>
       </c>
       <c r="H59" s="30" t="n">
-        <v>10.9</v>
+        <v>4.1</v>
       </c>
       <c r="I59" s="30" t="n">
-        <v>566</v>
+        <v>213</v>
       </c>
       <c r="J59" s="30" t="n">
-        <v>0</v>
+        <v>9.1</v>
       </c>
       <c r="K59" s="30" t="n">
-        <v>0</v>
+        <v>468</v>
       </c>
       <c r="L59" s="30" t="n">
         <v>46.1</v>
@@ -11291,22 +11291,22 @@
         <v>42</v>
       </c>
       <c r="F60" s="30" t="n">
-        <v>66.5</v>
+        <v>62.1</v>
       </c>
       <c r="G60" s="30" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="H60" s="30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I60" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="J60" s="30" t="n">
         <v>1.8</v>
       </c>
-      <c r="I60" s="30" t="n">
+      <c r="K60" s="30" t="n">
         <v>2</v>
-      </c>
-      <c r="J60" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" s="30" t="n">
-        <v>0</v>
       </c>
       <c r="L60" s="30" t="n">
         <v>68.3</v>
@@ -11469,22 +11469,22 @@
         <v>974</v>
       </c>
       <c r="F61" s="30" t="n">
-        <v>42.8</v>
+        <v>30.3</v>
       </c>
       <c r="G61" s="30" t="n">
-        <v>1752</v>
+        <v>1241</v>
       </c>
       <c r="H61" s="30" t="n">
-        <v>33.5</v>
+        <v>13</v>
       </c>
       <c r="I61" s="30" t="n">
-        <v>1371</v>
+        <v>533</v>
       </c>
       <c r="J61" s="30" t="n">
-        <v>0</v>
+        <v>32.9</v>
       </c>
       <c r="K61" s="30" t="n">
-        <v>0</v>
+        <v>1350</v>
       </c>
       <c r="L61" s="30" t="n">
         <v>76.2</v>
@@ -11494,7 +11494,7 @@
       </c>
       <c r="N61" s="31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O61" s="32" t="n">
@@ -11843,22 +11843,22 @@
         <v>234</v>
       </c>
       <c r="F63" s="30" t="n">
-        <v>42.3</v>
+        <v>25.4</v>
       </c>
       <c r="G63" s="30" t="n">
-        <v>234</v>
+        <v>140</v>
       </c>
       <c r="H63" s="30" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="I63" s="30" t="n">
+        <v>101</v>
+      </c>
+      <c r="J63" s="30" t="n">
         <v>14.1</v>
       </c>
-      <c r="I63" s="30" t="n">
+      <c r="K63" s="30" t="n">
         <v>78</v>
-      </c>
-      <c r="J63" s="30" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K63" s="30" t="n">
-        <v>8</v>
       </c>
       <c r="L63" s="30" t="n">
         <v>57.7</v>
@@ -11868,7 +11868,7 @@
       </c>
       <c r="N63" s="31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O63" s="32" t="n">
@@ -12391,34 +12391,34 @@
         <v>35114</v>
       </c>
       <c r="D66" s="30" t="n">
-        <v>69.8</v>
+        <v>58.2</v>
       </c>
       <c r="E66" s="30" t="n">
-        <v>24495</v>
+        <v>20435</v>
       </c>
       <c r="F66" s="30" t="n">
-        <v>23.2</v>
+        <v>33.4</v>
       </c>
       <c r="G66" s="30" t="n">
-        <v>8133</v>
+        <v>11723</v>
       </c>
       <c r="H66" s="30" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I66" s="30" t="n">
+        <v>540</v>
+      </c>
+      <c r="J66" s="30" t="n">
         <v>6.9</v>
       </c>
-      <c r="I66" s="30" t="n">
+      <c r="K66" s="30" t="n">
         <v>2416</v>
       </c>
-      <c r="J66" s="30" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K66" s="30" t="n">
-        <v>70</v>
-      </c>
       <c r="L66" s="30" t="n">
-        <v>30.2</v>
+        <v>41.8</v>
       </c>
       <c r="M66" s="30" t="n">
-        <v>10619</v>
+        <v>14679</v>
       </c>
       <c r="N66" s="31" t="inlineStr">
         <is>

</xml_diff>